<commit_message>
Add doctor appointment confirmation email to patients, manual operations for booking, review to post for doctors after appointment by patients
</commit_message>
<xml_diff>
--- a/generated_credentials.csv.xlsx
+++ b/generated_credentials.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DevProjects\Python\New folder\PH-ITI-W1T1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C64C2D46-5ED9-4416-9F64-ADF3007263AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F371D07B-66F3-487F-A081-BB743B574109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{3C734844-21FB-49C1-AB5D-A0AEA303718E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3C734844-21FB-49C1-AB5D-A0AEA303718E}"/>
   </bookViews>
   <sheets>
     <sheet name="generated_credentials" sheetId="1" r:id="rId1"/>
@@ -1186,16 +1186,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F09151C5-EE26-4E3B-8F6C-B34505F337C0}">
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1249,7 +1249,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1266,7 +1266,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1317,7 +1317,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -1487,7 +1487,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>54</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>54</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>54</v>
       </c>

</xml_diff>

<commit_message>
Added calendar changes and email capablities, added new Calendarlegend and status filse and react-icons dependency and final testing conditions regarding email for appointment cancellations and transfers
</commit_message>
<xml_diff>
--- a/generated_credentials.csv.xlsx
+++ b/generated_credentials.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4CD069-B533-4638-AA68-69BCF5849911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D78F86-01AD-4BCB-B82F-72E6DCAF9C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3C734844-21FB-49C1-AB5D-A0AEA303718E}"/>
   </bookViews>
@@ -1517,7 +1517,7 @@
       <c r="E19" t="s">
         <v>69</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1643,6 +1643,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D26" r:id="rId1" xr:uid="{80DAF278-EBC1-44A4-A070-9F58696A8F80}"/>
+    <hyperlink ref="F19" r:id="rId2" xr:uid="{B18AE106-8EAD-46CC-BDD5-36546E23E75B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NLP language detection (English/Roman Urdu/Native Urdu), update chat_router with hybrid NLP+LLM system, and improve multilingual support
</commit_message>
<xml_diff>
--- a/generated_credentials.csv.xlsx
+++ b/generated_credentials.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D78F86-01AD-4BCB-B82F-72E6DCAF9C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2EDE95-F5AD-46D8-B0DE-7C005FD02409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3C734844-21FB-49C1-AB5D-A0AEA303718E}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="107">
   <si>
     <t>role</t>
   </si>
@@ -314,6 +314,33 @@
   </si>
   <si>
     <t>alan1234</t>
+  </si>
+  <si>
+    <t>Admin101</t>
+  </si>
+  <si>
+    <t>ad101min</t>
+  </si>
+  <si>
+    <t>zubair019r</t>
+  </si>
+  <si>
+    <t>zubair019</t>
+  </si>
+  <si>
+    <t>zahmad28@gmail.com</t>
+  </si>
+  <si>
+    <t>sadia9191</t>
+  </si>
+  <si>
+    <t>sadia91919</t>
+  </si>
+  <si>
+    <t>Zubair Ahmed</t>
+  </si>
+  <si>
+    <t>Sadia Raza</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F09151C5-EE26-4E3B-8F6C-B34505F337C0}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
@@ -1640,10 +1667,53 @@
         <v>97</v>
       </c>
     </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E27" t="s">
+        <v>98</v>
+      </c>
+      <c r="F27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" t="s">
+        <v>105</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E28" t="s">
+        <v>101</v>
+      </c>
+      <c r="F28" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>103</v>
+      </c>
+      <c r="F29" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D26" r:id="rId1" xr:uid="{80DAF278-EBC1-44A4-A070-9F58696A8F80}"/>
     <hyperlink ref="F19" r:id="rId2" xr:uid="{B18AE106-8EAD-46CC-BDD5-36546E23E75B}"/>
+    <hyperlink ref="D28" r:id="rId3" xr:uid="{36EFFA2B-D124-4FEB-99A9-6D76C80B07C6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed UTC timing zone error for Admin controlling Patient Booking & allowed admin to set doctor image and open availability periods for patient appointments
</commit_message>
<xml_diff>
--- a/generated_credentials.csv.xlsx
+++ b/generated_credentials.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2EDE95-F5AD-46D8-B0DE-7C005FD02409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DABBB6-F432-468E-BD83-6A0AC9725B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3C734844-21FB-49C1-AB5D-A0AEA303718E}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="104">
   <si>
     <t>role</t>
   </si>
@@ -331,16 +331,7 @@
     <t>zahmad28@gmail.com</t>
   </si>
   <si>
-    <t>sadia9191</t>
-  </si>
-  <si>
-    <t>sadia91919</t>
-  </si>
-  <si>
     <t>Zubair Ahmed</t>
-  </si>
-  <si>
-    <t>Sadia Raza</t>
   </si>
 </sst>
 </file>
@@ -1212,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F09151C5-EE26-4E3B-8F6C-B34505F337C0}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
@@ -1680,7 +1671,7 @@
         <v>54</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>102</v>
@@ -1690,23 +1681,6 @@
       </c>
       <c r="F28" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" t="s">
-        <v>106</v>
-      </c>
-      <c r="C29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>103</v>
-      </c>
-      <c r="F29" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>